<commit_message>
major refactor — transform project from invoice tool to global document extraction system
</commit_message>
<xml_diff>
--- a/data/sample_invoice.xlsx
+++ b/data/sample_invoice.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danad\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danad\Desktop\Benim\Tutorials\Python\ocr-ai-extractor\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DE04D2A-0F0B-441A-8770-CE984115D395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{307D2879-A722-4D7B-AB87-85021F433A96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1050,6 +1050,9 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1059,162 +1062,180 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="12" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="10" fontId="3" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="4" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="3" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="3" fillId="4" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1268,27 +1289,6 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="12" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1619,133 +1619,133 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="60.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="70" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
-      <c r="E1" s="65"/>
-      <c r="F1" s="65"/>
-      <c r="G1" s="65"/>
-      <c r="H1" s="65"/>
-      <c r="I1" s="65"/>
-      <c r="J1" s="66"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="76" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="71"/>
-      <c r="C2" s="71"/>
-      <c r="D2" s="71"/>
-      <c r="E2" s="71"/>
-      <c r="F2" s="71"/>
-      <c r="G2" s="71"/>
-      <c r="H2" s="71"/>
-      <c r="I2" s="71"/>
-      <c r="J2" s="72"/>
+      <c r="B2" s="77"/>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
+      <c r="F2" s="77"/>
+      <c r="G2" s="77"/>
+      <c r="H2" s="77"/>
+      <c r="I2" s="77"/>
+      <c r="J2" s="78"/>
     </row>
     <row r="3" spans="1:13" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="73"/>
-      <c r="B3" s="74"/>
-      <c r="C3" s="74"/>
-      <c r="D3" s="74"/>
-      <c r="E3" s="74"/>
-      <c r="F3" s="74"/>
-      <c r="G3" s="74"/>
-      <c r="H3" s="74"/>
-      <c r="I3" s="74"/>
-      <c r="J3" s="75"/>
+      <c r="A3" s="79"/>
+      <c r="B3" s="80"/>
+      <c r="C3" s="80"/>
+      <c r="D3" s="80"/>
+      <c r="E3" s="80"/>
+      <c r="F3" s="80"/>
+      <c r="G3" s="80"/>
+      <c r="H3" s="80"/>
+      <c r="I3" s="80"/>
+      <c r="J3" s="81"/>
     </row>
     <row r="4" spans="1:13" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="76"/>
-      <c r="B4" s="77"/>
-      <c r="C4" s="77"/>
-      <c r="D4" s="77"/>
-      <c r="E4" s="77"/>
-      <c r="F4" s="77"/>
-      <c r="G4" s="77"/>
-      <c r="H4" s="77"/>
-      <c r="I4" s="77"/>
-      <c r="J4" s="78"/>
+      <c r="A4" s="83"/>
+      <c r="B4" s="84"/>
+      <c r="C4" s="84"/>
+      <c r="D4" s="84"/>
+      <c r="E4" s="84"/>
+      <c r="F4" s="84"/>
+      <c r="G4" s="84"/>
+      <c r="H4" s="84"/>
+      <c r="I4" s="84"/>
+      <c r="J4" s="85"/>
     </row>
     <row r="5" spans="1:13" ht="30.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="67" t="s">
+      <c r="A5" s="73" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="68"/>
-      <c r="C5" s="68"/>
-      <c r="D5" s="68"/>
-      <c r="E5" s="68"/>
-      <c r="F5" s="68"/>
-      <c r="G5" s="68"/>
-      <c r="H5" s="68"/>
-      <c r="I5" s="68"/>
-      <c r="J5" s="69"/>
+      <c r="B5" s="74"/>
+      <c r="C5" s="74"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="74"/>
+      <c r="F5" s="74"/>
+      <c r="G5" s="74"/>
+      <c r="H5" s="74"/>
+      <c r="I5" s="74"/>
+      <c r="J5" s="75"/>
     </row>
     <row r="6" spans="1:13" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="24"/>
-      <c r="C6" s="24"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="53" t="s">
+      <c r="B6" s="60"/>
+      <c r="C6" s="60"/>
+      <c r="D6" s="60"/>
+      <c r="E6" s="60"/>
+      <c r="F6" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="53"/>
-      <c r="H6" s="24"/>
-      <c r="I6" s="24"/>
-      <c r="J6" s="24"/>
+      <c r="G6" s="58"/>
+      <c r="H6" s="60"/>
+      <c r="I6" s="60"/>
+      <c r="J6" s="60"/>
     </row>
     <row r="7" spans="1:13" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="25"/>
-      <c r="C7" s="25"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
-      <c r="F7" s="54" t="s">
+      <c r="B7" s="82"/>
+      <c r="C7" s="82"/>
+      <c r="D7" s="82"/>
+      <c r="E7" s="82"/>
+      <c r="F7" s="59" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="54"/>
-      <c r="H7" s="25"/>
-      <c r="I7" s="25"/>
-      <c r="J7" s="25"/>
+      <c r="G7" s="59"/>
+      <c r="H7" s="82"/>
+      <c r="I7" s="82"/>
+      <c r="J7" s="82"/>
     </row>
     <row r="8" spans="1:13" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="25"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="25"/>
-      <c r="E8" s="25"/>
-      <c r="F8" s="54" t="s">
+      <c r="B8" s="82"/>
+      <c r="C8" s="82"/>
+      <c r="D8" s="82"/>
+      <c r="E8" s="82"/>
+      <c r="F8" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="G8" s="54"/>
-      <c r="H8" s="25"/>
-      <c r="I8" s="25"/>
-      <c r="J8" s="25"/>
+      <c r="G8" s="59"/>
+      <c r="H8" s="82"/>
+      <c r="I8" s="82"/>
+      <c r="J8" s="82"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
     </row>
     <row r="9" spans="1:13" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="89"/>
-      <c r="B9" s="90"/>
-      <c r="C9" s="90"/>
-      <c r="D9" s="90"/>
-      <c r="E9" s="90"/>
-      <c r="F9" s="90"/>
-      <c r="G9" s="90"/>
-      <c r="H9" s="90"/>
-      <c r="I9" s="90"/>
-      <c r="J9" s="91"/>
+      <c r="A9" s="96"/>
+      <c r="B9" s="97"/>
+      <c r="C9" s="97"/>
+      <c r="D9" s="97"/>
+      <c r="E9" s="97"/>
+      <c r="F9" s="97"/>
+      <c r="G9" s="97"/>
+      <c r="H9" s="97"/>
+      <c r="I9" s="97"/>
+      <c r="J9" s="98"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
@@ -1754,17 +1754,17 @@
       <c r="A10" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="92" t="s">
+      <c r="B10" s="99" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="92"/>
-      <c r="D10" s="92"/>
-      <c r="E10" s="92"/>
-      <c r="F10" s="92"/>
-      <c r="G10" s="92"/>
-      <c r="H10" s="92"/>
-      <c r="I10" s="92"/>
-      <c r="J10" s="93"/>
+      <c r="C10" s="99"/>
+      <c r="D10" s="99"/>
+      <c r="E10" s="99"/>
+      <c r="F10" s="99"/>
+      <c r="G10" s="99"/>
+      <c r="H10" s="99"/>
+      <c r="I10" s="99"/>
+      <c r="J10" s="100"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
@@ -1773,27 +1773,27 @@
       <c r="A11" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="96" t="s">
+      <c r="B11" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="97" t="s">
+      <c r="C11" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="97" t="s">
+      <c r="D11" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="E11" s="98" t="s">
+      <c r="E11" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="F11" s="53" t="s">
+      <c r="F11" s="58" t="s">
         <v>21</v>
       </c>
-      <c r="G11" s="53"/>
-      <c r="H11" s="24">
+      <c r="G11" s="58"/>
+      <c r="H11" s="60">
         <v>425798</v>
       </c>
-      <c r="I11" s="24"/>
-      <c r="J11" s="24"/>
+      <c r="I11" s="60"/>
+      <c r="J11" s="60"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
@@ -1802,25 +1802,25 @@
       <c r="A12" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="99">
+      <c r="B12" s="28">
         <v>46153</v>
       </c>
-      <c r="C12" s="94">
+      <c r="C12" s="29">
         <v>46153</v>
       </c>
-      <c r="D12" s="94">
+      <c r="D12" s="29">
         <v>46153</v>
       </c>
-      <c r="E12" s="95">
+      <c r="E12" s="30">
         <v>46153</v>
       </c>
-      <c r="F12" s="54" t="s">
+      <c r="F12" s="59" t="s">
         <v>12</v>
       </c>
-      <c r="G12" s="54"/>
-      <c r="H12" s="25"/>
-      <c r="I12" s="25"/>
-      <c r="J12" s="25"/>
+      <c r="G12" s="59"/>
+      <c r="H12" s="82"/>
+      <c r="I12" s="82"/>
+      <c r="J12" s="82"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
@@ -1829,40 +1829,40 @@
       <c r="A13" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="99">
+      <c r="B13" s="28">
         <v>46162</v>
       </c>
-      <c r="C13" s="94">
+      <c r="C13" s="29">
         <v>4473274</v>
       </c>
-      <c r="D13" s="94">
+      <c r="D13" s="29">
         <v>4473274</v>
       </c>
-      <c r="E13" s="95">
+      <c r="E13" s="30">
         <v>4473274</v>
       </c>
-      <c r="F13" s="54" t="s">
+      <c r="F13" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="G13" s="54"/>
-      <c r="H13" s="25"/>
-      <c r="I13" s="25"/>
-      <c r="J13" s="25"/>
+      <c r="G13" s="59"/>
+      <c r="H13" s="82"/>
+      <c r="I13" s="82"/>
+      <c r="J13" s="82"/>
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
     </row>
     <row r="14" spans="1:13" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="35"/>
-      <c r="B14" s="36"/>
-      <c r="C14" s="36"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="36"/>
-      <c r="F14" s="36"/>
-      <c r="G14" s="36"/>
-      <c r="H14" s="36"/>
-      <c r="I14" s="36"/>
-      <c r="J14" s="37"/>
+      <c r="A14" s="40"/>
+      <c r="B14" s="41"/>
+      <c r="C14" s="41"/>
+      <c r="D14" s="41"/>
+      <c r="E14" s="41"/>
+      <c r="F14" s="41"/>
+      <c r="G14" s="41"/>
+      <c r="H14" s="41"/>
+      <c r="I14" s="41"/>
+      <c r="J14" s="42"/>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
@@ -1874,20 +1874,20 @@
       <c r="B15" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C15" s="81" t="s">
+      <c r="C15" s="88" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="82"/>
-      <c r="E15" s="82"/>
-      <c r="F15" s="82"/>
-      <c r="G15" s="83"/>
+      <c r="D15" s="89"/>
+      <c r="E15" s="89"/>
+      <c r="F15" s="89"/>
+      <c r="G15" s="90"/>
       <c r="H15" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="84" t="s">
+      <c r="I15" s="91" t="s">
         <v>4</v>
       </c>
-      <c r="J15" s="85"/>
+      <c r="J15" s="92"/>
       <c r="K15" s="1"/>
     </row>
     <row r="16" spans="1:13" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
@@ -1897,21 +1897,21 @@
       <c r="B16" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="86" t="s">
+      <c r="C16" s="93" t="s">
         <v>29</v>
       </c>
-      <c r="D16" s="87"/>
-      <c r="E16" s="87"/>
-      <c r="F16" s="87"/>
-      <c r="G16" s="88"/>
+      <c r="D16" s="94"/>
+      <c r="E16" s="94"/>
+      <c r="F16" s="94"/>
+      <c r="G16" s="95"/>
       <c r="H16" s="15">
         <v>1200</v>
       </c>
-      <c r="I16" s="38">
+      <c r="I16" s="43">
         <f>($A16*$H16)</f>
         <v>1200</v>
       </c>
-      <c r="J16" s="39"/>
+      <c r="J16" s="44"/>
       <c r="K16" s="1"/>
     </row>
     <row r="17" spans="1:13" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
@@ -1921,21 +1921,21 @@
       <c r="B17" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C17" s="40" t="s">
+      <c r="C17" s="45" t="s">
         <v>30</v>
       </c>
-      <c r="D17" s="41"/>
-      <c r="E17" s="41"/>
-      <c r="F17" s="41"/>
-      <c r="G17" s="42"/>
+      <c r="D17" s="46"/>
+      <c r="E17" s="46"/>
+      <c r="F17" s="46"/>
+      <c r="G17" s="47"/>
       <c r="H17" s="16">
         <v>25</v>
       </c>
-      <c r="I17" s="79">
-        <f t="shared" ref="I17:I33" si="0">($A17*$H17)</f>
+      <c r="I17" s="86">
+        <f t="shared" ref="I17:I18" si="0">($A17*$H17)</f>
         <v>50</v>
       </c>
-      <c r="J17" s="80"/>
+      <c r="J17" s="87"/>
       <c r="K17" s="1"/>
     </row>
     <row r="18" spans="1:13" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
@@ -1945,99 +1945,99 @@
       <c r="B18" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="C18" s="45" t="s">
+      <c r="C18" s="50" t="s">
         <v>31</v>
       </c>
-      <c r="D18" s="46"/>
-      <c r="E18" s="46"/>
-      <c r="F18" s="46"/>
-      <c r="G18" s="47"/>
+      <c r="D18" s="51"/>
+      <c r="E18" s="51"/>
+      <c r="F18" s="51"/>
+      <c r="G18" s="52"/>
       <c r="H18" s="17">
         <v>45</v>
       </c>
-      <c r="I18" s="38">
+      <c r="I18" s="43">
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
-      <c r="J18" s="39"/>
+      <c r="J18" s="44"/>
       <c r="K18" s="1"/>
     </row>
     <row r="19" spans="1:13" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="9"/>
       <c r="B19" s="10"/>
-      <c r="C19" s="40"/>
-      <c r="D19" s="41"/>
-      <c r="E19" s="41"/>
-      <c r="F19" s="41"/>
-      <c r="G19" s="42"/>
+      <c r="C19" s="45"/>
+      <c r="D19" s="46"/>
+      <c r="E19" s="46"/>
+      <c r="F19" s="46"/>
+      <c r="G19" s="47"/>
       <c r="H19" s="16"/>
-      <c r="I19" s="43"/>
-      <c r="J19" s="44"/>
+      <c r="I19" s="48"/>
+      <c r="J19" s="49"/>
       <c r="K19" s="1"/>
     </row>
     <row r="20" spans="1:13" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="11"/>
       <c r="B20" s="12"/>
-      <c r="C20" s="45"/>
-      <c r="D20" s="46"/>
-      <c r="E20" s="46"/>
-      <c r="F20" s="46"/>
-      <c r="G20" s="47"/>
+      <c r="C20" s="50"/>
+      <c r="D20" s="51"/>
+      <c r="E20" s="51"/>
+      <c r="F20" s="51"/>
+      <c r="G20" s="52"/>
       <c r="H20" s="17"/>
-      <c r="I20" s="38"/>
-      <c r="J20" s="39"/>
+      <c r="I20" s="43"/>
+      <c r="J20" s="44"/>
       <c r="K20" s="1"/>
     </row>
     <row r="21" spans="1:13" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="9"/>
       <c r="B21" s="10"/>
-      <c r="C21" s="40"/>
-      <c r="D21" s="41"/>
-      <c r="E21" s="41"/>
-      <c r="F21" s="41"/>
-      <c r="G21" s="42"/>
+      <c r="C21" s="45"/>
+      <c r="D21" s="46"/>
+      <c r="E21" s="46"/>
+      <c r="F21" s="46"/>
+      <c r="G21" s="47"/>
       <c r="H21" s="16"/>
-      <c r="I21" s="43"/>
-      <c r="J21" s="44"/>
+      <c r="I21" s="48"/>
+      <c r="J21" s="49"/>
       <c r="K21" s="1"/>
     </row>
     <row r="22" spans="1:13" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="11"/>
       <c r="B22" s="12"/>
-      <c r="C22" s="45"/>
-      <c r="D22" s="46"/>
-      <c r="E22" s="46"/>
-      <c r="F22" s="46"/>
-      <c r="G22" s="47"/>
+      <c r="C22" s="50"/>
+      <c r="D22" s="51"/>
+      <c r="E22" s="51"/>
+      <c r="F22" s="51"/>
+      <c r="G22" s="52"/>
       <c r="H22" s="17"/>
-      <c r="I22" s="38"/>
-      <c r="J22" s="39"/>
+      <c r="I22" s="43"/>
+      <c r="J22" s="44"/>
       <c r="K22" s="1"/>
     </row>
     <row r="23" spans="1:13" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="9"/>
       <c r="B23" s="10"/>
-      <c r="C23" s="40"/>
-      <c r="D23" s="41"/>
-      <c r="E23" s="41"/>
-      <c r="F23" s="41"/>
-      <c r="G23" s="42"/>
+      <c r="C23" s="45"/>
+      <c r="D23" s="46"/>
+      <c r="E23" s="46"/>
+      <c r="F23" s="46"/>
+      <c r="G23" s="47"/>
       <c r="H23" s="16"/>
-      <c r="I23" s="43"/>
-      <c r="J23" s="44"/>
+      <c r="I23" s="48"/>
+      <c r="J23" s="49"/>
       <c r="K23" s="1"/>
     </row>
     <row r="24" spans="1:13" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="11"/>
       <c r="B24" s="12"/>
-      <c r="C24" s="45"/>
-      <c r="D24" s="46"/>
-      <c r="E24" s="46"/>
-      <c r="F24" s="46"/>
-      <c r="G24" s="47"/>
+      <c r="C24" s="50"/>
+      <c r="D24" s="51"/>
+      <c r="E24" s="51"/>
+      <c r="F24" s="51"/>
+      <c r="G24" s="52"/>
       <c r="H24" s="17"/>
-      <c r="I24" s="38"/>
-      <c r="J24" s="39"/>
+      <c r="I24" s="43"/>
+      <c r="J24" s="44"/>
       <c r="K24" s="1"/>
       <c r="L24" s="1"/>
       <c r="M24" s="1"/>
@@ -2045,14 +2045,14 @@
     <row r="25" spans="1:13" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="9"/>
       <c r="B25" s="10"/>
-      <c r="C25" s="40"/>
-      <c r="D25" s="41"/>
-      <c r="E25" s="41"/>
-      <c r="F25" s="41"/>
-      <c r="G25" s="42"/>
+      <c r="C25" s="45"/>
+      <c r="D25" s="46"/>
+      <c r="E25" s="46"/>
+      <c r="F25" s="46"/>
+      <c r="G25" s="47"/>
       <c r="H25" s="16"/>
-      <c r="I25" s="43"/>
-      <c r="J25" s="44"/>
+      <c r="I25" s="48"/>
+      <c r="J25" s="49"/>
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
       <c r="M25" s="1"/>
@@ -2060,14 +2060,14 @@
     <row r="26" spans="1:13" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="11"/>
       <c r="B26" s="12"/>
-      <c r="C26" s="45"/>
-      <c r="D26" s="46"/>
-      <c r="E26" s="46"/>
-      <c r="F26" s="46"/>
-      <c r="G26" s="47"/>
+      <c r="C26" s="50"/>
+      <c r="D26" s="51"/>
+      <c r="E26" s="51"/>
+      <c r="F26" s="51"/>
+      <c r="G26" s="52"/>
       <c r="H26" s="17"/>
-      <c r="I26" s="38"/>
-      <c r="J26" s="39"/>
+      <c r="I26" s="43"/>
+      <c r="J26" s="44"/>
       <c r="K26" s="1"/>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
@@ -2075,14 +2075,14 @@
     <row r="27" spans="1:13" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="9"/>
       <c r="B27" s="10"/>
-      <c r="C27" s="40"/>
-      <c r="D27" s="41"/>
-      <c r="E27" s="41"/>
-      <c r="F27" s="41"/>
-      <c r="G27" s="42"/>
+      <c r="C27" s="45"/>
+      <c r="D27" s="46"/>
+      <c r="E27" s="46"/>
+      <c r="F27" s="46"/>
+      <c r="G27" s="47"/>
       <c r="H27" s="16"/>
-      <c r="I27" s="43"/>
-      <c r="J27" s="44"/>
+      <c r="I27" s="48"/>
+      <c r="J27" s="49"/>
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
@@ -2090,14 +2090,14 @@
     <row r="28" spans="1:13" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="11"/>
       <c r="B28" s="12"/>
-      <c r="C28" s="45"/>
-      <c r="D28" s="46"/>
-      <c r="E28" s="46"/>
-      <c r="F28" s="46"/>
-      <c r="G28" s="47"/>
+      <c r="C28" s="50"/>
+      <c r="D28" s="51"/>
+      <c r="E28" s="51"/>
+      <c r="F28" s="51"/>
+      <c r="G28" s="52"/>
       <c r="H28" s="17"/>
-      <c r="I28" s="38"/>
-      <c r="J28" s="39"/>
+      <c r="I28" s="43"/>
+      <c r="J28" s="44"/>
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
@@ -2105,14 +2105,14 @@
     <row r="29" spans="1:13" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="9"/>
       <c r="B29" s="10"/>
-      <c r="C29" s="40"/>
-      <c r="D29" s="41"/>
-      <c r="E29" s="41"/>
-      <c r="F29" s="41"/>
-      <c r="G29" s="42"/>
+      <c r="C29" s="45"/>
+      <c r="D29" s="46"/>
+      <c r="E29" s="46"/>
+      <c r="F29" s="46"/>
+      <c r="G29" s="47"/>
       <c r="H29" s="16"/>
-      <c r="I29" s="43"/>
-      <c r="J29" s="44"/>
+      <c r="I29" s="48"/>
+      <c r="J29" s="49"/>
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
@@ -2120,14 +2120,14 @@
     <row r="30" spans="1:13" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="11"/>
       <c r="B30" s="12"/>
-      <c r="C30" s="45"/>
-      <c r="D30" s="46"/>
-      <c r="E30" s="46"/>
-      <c r="F30" s="46"/>
-      <c r="G30" s="47"/>
+      <c r="C30" s="50"/>
+      <c r="D30" s="51"/>
+      <c r="E30" s="51"/>
+      <c r="F30" s="51"/>
+      <c r="G30" s="52"/>
       <c r="H30" s="17"/>
-      <c r="I30" s="38"/>
-      <c r="J30" s="39"/>
+      <c r="I30" s="43"/>
+      <c r="J30" s="44"/>
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
@@ -2135,14 +2135,14 @@
     <row r="31" spans="1:13" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="9"/>
       <c r="B31" s="10"/>
-      <c r="C31" s="40"/>
-      <c r="D31" s="41"/>
-      <c r="E31" s="41"/>
-      <c r="F31" s="41"/>
-      <c r="G31" s="42"/>
+      <c r="C31" s="45"/>
+      <c r="D31" s="46"/>
+      <c r="E31" s="46"/>
+      <c r="F31" s="46"/>
+      <c r="G31" s="47"/>
       <c r="H31" s="16"/>
-      <c r="I31" s="43"/>
-      <c r="J31" s="44"/>
+      <c r="I31" s="48"/>
+      <c r="J31" s="49"/>
       <c r="K31" s="1"/>
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
@@ -2150,14 +2150,14 @@
     <row r="32" spans="1:13" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="11"/>
       <c r="B32" s="12"/>
-      <c r="C32" s="45"/>
-      <c r="D32" s="46"/>
-      <c r="E32" s="46"/>
-      <c r="F32" s="46"/>
-      <c r="G32" s="47"/>
+      <c r="C32" s="50"/>
+      <c r="D32" s="51"/>
+      <c r="E32" s="51"/>
+      <c r="F32" s="51"/>
+      <c r="G32" s="52"/>
       <c r="H32" s="17"/>
-      <c r="I32" s="38"/>
-      <c r="J32" s="39"/>
+      <c r="I32" s="43"/>
+      <c r="J32" s="44"/>
       <c r="K32" s="1"/>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
@@ -2165,111 +2165,111 @@
     <row r="33" spans="1:13" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="13"/>
       <c r="B33" s="14"/>
-      <c r="C33" s="59"/>
-      <c r="D33" s="60"/>
-      <c r="E33" s="60"/>
-      <c r="F33" s="60"/>
-      <c r="G33" s="61"/>
+      <c r="C33" s="65"/>
+      <c r="D33" s="66"/>
+      <c r="E33" s="66"/>
+      <c r="F33" s="66"/>
+      <c r="G33" s="67"/>
       <c r="H33" s="16"/>
-      <c r="I33" s="43"/>
-      <c r="J33" s="44"/>
+      <c r="I33" s="48"/>
+      <c r="J33" s="49"/>
       <c r="K33" s="1"/>
       <c r="L33" s="1"/>
       <c r="M33" s="1"/>
     </row>
     <row r="34" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="26" t="s">
+      <c r="A34" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="B34" s="27"/>
-      <c r="C34" s="27"/>
-      <c r="D34" s="27"/>
-      <c r="E34" s="27"/>
-      <c r="F34" s="27"/>
-      <c r="G34" s="28"/>
+      <c r="B34" s="32"/>
+      <c r="C34" s="32"/>
+      <c r="D34" s="32"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="32"/>
+      <c r="G34" s="33"/>
       <c r="H34" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="I34" s="62">
+      <c r="I34" s="68">
         <f>SUM(I16:J33)</f>
         <v>1295</v>
       </c>
-      <c r="J34" s="63"/>
+      <c r="J34" s="69"/>
       <c r="K34" s="1"/>
       <c r="L34" s="1"/>
       <c r="M34" s="1"/>
     </row>
     <row r="35" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="29"/>
-      <c r="B35" s="30"/>
-      <c r="C35" s="30"/>
-      <c r="D35" s="30"/>
-      <c r="E35" s="30"/>
-      <c r="F35" s="30"/>
-      <c r="G35" s="31"/>
+      <c r="A35" s="34"/>
+      <c r="B35" s="35"/>
+      <c r="C35" s="35"/>
+      <c r="D35" s="35"/>
+      <c r="E35" s="35"/>
+      <c r="F35" s="35"/>
+      <c r="G35" s="36"/>
       <c r="H35" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="I35" s="55">
+      <c r="I35" s="61">
         <v>0.1</v>
       </c>
-      <c r="J35" s="56"/>
+      <c r="J35" s="62"/>
       <c r="K35" s="1"/>
       <c r="L35" s="1"/>
       <c r="M35" s="1"/>
     </row>
     <row r="36" spans="1:13" ht="26.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="32"/>
-      <c r="B36" s="33"/>
-      <c r="C36" s="33"/>
-      <c r="D36" s="33"/>
-      <c r="E36" s="33"/>
-      <c r="F36" s="33"/>
-      <c r="G36" s="34"/>
+      <c r="A36" s="37"/>
+      <c r="B36" s="38"/>
+      <c r="C36" s="38"/>
+      <c r="D36" s="38"/>
+      <c r="E36" s="38"/>
+      <c r="F36" s="38"/>
+      <c r="G36" s="39"/>
       <c r="H36" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="I36" s="57">
+      <c r="I36" s="63">
         <f>I34*(1+I35)</f>
         <v>1424.5000000000002</v>
       </c>
-      <c r="J36" s="58"/>
+      <c r="J36" s="64"/>
       <c r="K36" s="1"/>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
     </row>
     <row r="37" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="51" t="s">
+      <c r="A37" s="56" t="s">
         <v>7</v>
       </c>
-      <c r="B37" s="52"/>
-      <c r="C37" s="52"/>
-      <c r="D37" s="52"/>
-      <c r="E37" s="52"/>
-      <c r="F37" s="100">
+      <c r="B37" s="57"/>
+      <c r="C37" s="57"/>
+      <c r="D37" s="57"/>
+      <c r="E37" s="57"/>
+      <c r="F37" s="21">
         <v>7</v>
       </c>
-      <c r="G37" s="21"/>
-      <c r="H37" s="22"/>
-      <c r="I37" s="22"/>
-      <c r="J37" s="23"/>
+      <c r="G37" s="22"/>
+      <c r="H37" s="23"/>
+      <c r="I37" s="23"/>
+      <c r="J37" s="24"/>
       <c r="K37" s="1"/>
       <c r="L37" s="1"/>
       <c r="M37" s="1"/>
     </row>
     <row r="38" spans="1:13" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="48" t="s">
+      <c r="A38" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="B38" s="49"/>
-      <c r="C38" s="49"/>
-      <c r="D38" s="49"/>
-      <c r="E38" s="49"/>
-      <c r="F38" s="49"/>
-      <c r="G38" s="49"/>
-      <c r="H38" s="49"/>
-      <c r="I38" s="49"/>
-      <c r="J38" s="50"/>
+      <c r="B38" s="54"/>
+      <c r="C38" s="54"/>
+      <c r="D38" s="54"/>
+      <c r="E38" s="54"/>
+      <c r="F38" s="54"/>
+      <c r="G38" s="54"/>
+      <c r="H38" s="54"/>
+      <c r="I38" s="54"/>
+      <c r="J38" s="55"/>
       <c r="K38" s="1"/>
       <c r="L38" s="1"/>
       <c r="M38" s="1"/>

</xml_diff>